<commit_message>
Logged data for 27JUL26
</commit_message>
<xml_diff>
--- a/Marathon_Training_Log.xlsx
+++ b/Marathon_Training_Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prsap\Dropbox (Personal)\Personal\Marathon Training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Coursework\24-Git_Projects\02-Marathon_Training_Personal\Marathon_Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D9CA19E-2000-4942-AA0F-DE6512AB4371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9C8120-823B-4D29-A36A-74DFEFAD3694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="74">
   <si>
     <t>Marathon Training Log — Pre-Super Base</t>
   </si>
@@ -254,6 +254,12 @@
   </si>
   <si>
     <t>There are no pace targets in this block by design — run everything by feel. Pace/HR should be LOGGED for your own trend-tracking, not used as a target.</t>
+  </si>
+  <si>
+    <t>10 min Pre-Run Warm Up with Matt Wilpers + 30 min Tempo Run with Matt Wilpers</t>
+  </si>
+  <si>
+    <t>Completed additiona 35 min run with Apple watch. Heart rate did not actually reflect RPE. Slightly hot weather and mix of hills.</t>
   </si>
 </sst>
 </file>
@@ -369,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -417,6 +423,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -685,17 +697,19 @@
   <dimension ref="B2:P61"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="9" customWidth="1"/>
-    <col min="12" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="9" customWidth="1"/>
-    <col min="16" max="16" width="32" customWidth="1"/>
+    <col min="2" max="2" width="43.140625" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="111" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="71.5703125" customWidth="1"/>
+    <col min="8" max="8" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="43.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -703,11 +717,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="2:16" s="21" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="B3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="20" t="s">
         <v>2</v>
       </c>
     </row>
@@ -758,7 +772,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4">
         <v>46230</v>
       </c>
@@ -774,20 +788,36 @@
       <c r="F6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="7"/>
+      <c r="G6" s="7" t="s">
+        <v>72</v>
+      </c>
       <c r="H6" s="8" t="s">
         <v>21</v>
       </c>
       <c r="I6" s="5">
         <v>65</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="7"/>
+      <c r="J6" s="8">
+        <v>65</v>
+      </c>
+      <c r="K6" s="8">
+        <v>5.01</v>
+      </c>
+      <c r="L6" s="8">
+        <v>12.97</v>
+      </c>
+      <c r="M6" s="8">
+        <v>171</v>
+      </c>
+      <c r="N6" s="8">
+        <v>178</v>
+      </c>
+      <c r="O6" s="8">
+        <v>5</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="7" spans="2:16" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="9">
@@ -2554,11 +2584,11 @@
       </c>
       <c r="D6" s="15">
         <f>SUMIFS(Log!$J$6:$J$61,Log!$D$6:$D$61,B6)</f>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(Log!$K$6:$K$61,Log!$D$6:$D$61,B6)</f>
-        <v>0</v>
+        <v>5.01</v>
       </c>
       <c r="F6" s="15" t="str">
         <f>IFERROR(AVERAGEIFS(Log!$O$6:$O$61,Log!$D$6:$D$61,B6,Log!$H$6:$H$61,"Done"),"")</f>
@@ -2722,11 +2752,11 @@
       </c>
       <c r="D14" s="17">
         <f>SUM(D6:D13)</f>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E14" s="17">
         <f>SUM(E6:E13)</f>
-        <v>0</v>
+        <v>5.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated all remaining logs till 12AUG2026
</commit_message>
<xml_diff>
--- a/Marathon_Training_Log.xlsx
+++ b/Marathon_Training_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Coursework\24-Git_Projects\02-Marathon_Training_Personal\Marathon_Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1190F2A4-D578-4511-845D-27334B2C88D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B86BE2-D554-4372-A969-92E023529C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="102">
   <si>
     <t>Marathon Training Log — Pre-Super Base</t>
   </si>
@@ -306,7 +306,49 @@
     <t>Long walk with the dog to move around. No exersion at all.</t>
   </si>
   <si>
-    <t>Plan to finish the Strength class from week 1</t>
+    <t>Combination of 45 min Tempo Run with Becs Gentry + 10 min Pre-Run Warm Up with Matt Wilpers + 10 min cooldown</t>
+  </si>
+  <si>
+    <t>Actual run excluding WU and CD to be 45 matchign class. Distance 3.79 miles. Running behind by 1 day.</t>
+  </si>
+  <si>
+    <t>Did striders on Saturday bur un on 10AUG2026 Monday</t>
+  </si>
+  <si>
+    <t>Did long run this day.</t>
+  </si>
+  <si>
+    <t>30 min 2010s Run with Adrian Williams + 20 min run</t>
+  </si>
+  <si>
+    <t>45 min Marathon Race Prep with Robin Arzon + 10 min Pre run warmup</t>
+  </si>
+  <si>
+    <t>45 min Tempo Run with Becs Gentry  + 20 min run</t>
+  </si>
+  <si>
+    <t>30 min Strength for funners with Rebecca Kennedy</t>
+  </si>
+  <si>
+    <t>Strength training</t>
+  </si>
+  <si>
+    <t>Nose breathing run</t>
+  </si>
+  <si>
+    <t>Night walk</t>
+  </si>
+  <si>
+    <t>Just walk</t>
+  </si>
+  <si>
+    <t>Rested</t>
+  </si>
+  <si>
+    <t>Saturdays long run done this day. Too much hilly route. Definitely had to slow down.</t>
+  </si>
+  <si>
+    <t>Just did striders.</t>
   </si>
 </sst>
 </file>
@@ -1164,7 +1206,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>27</v>
@@ -1172,13 +1214,27 @@
       <c r="I13" s="14">
         <v>0</v>
       </c>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="8"/>
+      <c r="J13" s="9">
+        <v>30</v>
+      </c>
+      <c r="K13" s="9">
+        <v>0</v>
+      </c>
+      <c r="L13" s="9">
+        <v>0</v>
+      </c>
+      <c r="M13" s="9">
+        <v>120</v>
+      </c>
+      <c r="N13" s="9">
+        <v>155</v>
+      </c>
+      <c r="O13" s="9">
+        <v>3</v>
+      </c>
+      <c r="P13" s="8" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="14" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5">
@@ -1196,20 +1252,36 @@
       <c r="F14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>93</v>
+      </c>
       <c r="H14" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I14" s="6">
         <v>65</v>
       </c>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="8"/>
+      <c r="J14" s="9">
+        <v>65</v>
+      </c>
+      <c r="K14" s="9">
+        <v>4.87</v>
+      </c>
+      <c r="L14" s="9">
+        <v>12.55</v>
+      </c>
+      <c r="M14" s="9">
+        <v>153</v>
+      </c>
+      <c r="N14" s="9">
+        <v>165</v>
+      </c>
+      <c r="O14" s="9">
+        <v>5</v>
+      </c>
+      <c r="P14" s="8" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="15" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="10">
@@ -1227,20 +1299,36 @@
       <c r="F15" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="G15" s="8"/>
+      <c r="G15" s="8" t="s">
+        <v>92</v>
+      </c>
       <c r="H15" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I15" s="11">
         <v>52</v>
       </c>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="8"/>
+      <c r="J15" s="9">
+        <v>55</v>
+      </c>
+      <c r="K15" s="9">
+        <v>3.73</v>
+      </c>
+      <c r="L15" s="9">
+        <v>12.45</v>
+      </c>
+      <c r="M15" s="9">
+        <v>155</v>
+      </c>
+      <c r="N15" s="9">
+        <v>178</v>
+      </c>
+      <c r="O15" s="9">
+        <v>5</v>
+      </c>
+      <c r="P15" s="8" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="16" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="13">
@@ -1258,20 +1346,34 @@
       <c r="F16" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="8"/>
+      <c r="G16" s="8" t="s">
+        <v>97</v>
+      </c>
       <c r="H16" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I16" s="14">
         <v>0</v>
       </c>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
+      <c r="J16" s="9">
+        <v>22</v>
+      </c>
+      <c r="K16" s="9">
+        <v>0.86</v>
+      </c>
       <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="8"/>
+      <c r="M16" s="9">
+        <v>104</v>
+      </c>
+      <c r="N16" s="9">
+        <v>123</v>
+      </c>
+      <c r="O16" s="9">
+        <v>2</v>
+      </c>
+      <c r="P16" s="8" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="17" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="5">
@@ -1289,19 +1391,33 @@
       <c r="F17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G17" s="8"/>
+      <c r="G17" s="8" t="s">
+        <v>91</v>
+      </c>
       <c r="H17" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="6">
         <v>50</v>
       </c>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
+      <c r="J17" s="9">
+        <v>50</v>
+      </c>
+      <c r="K17" s="9">
+        <v>3.74</v>
+      </c>
+      <c r="L17" s="9">
+        <v>13.02</v>
+      </c>
+      <c r="M17" s="9">
+        <v>146</v>
+      </c>
+      <c r="N17" s="9">
+        <v>165</v>
+      </c>
+      <c r="O17" s="9">
+        <v>5</v>
+      </c>
       <c r="P17" s="8"/>
     </row>
     <row r="18" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1320,20 +1436,36 @@
       <c r="F18" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="8"/>
+      <c r="G18" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="H18" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I18" s="11">
         <v>135</v>
       </c>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="8"/>
+      <c r="J18" s="9">
+        <v>20</v>
+      </c>
+      <c r="K18" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="L18" s="9">
+        <v>14.13</v>
+      </c>
+      <c r="M18" s="9">
+        <v>145</v>
+      </c>
+      <c r="N18" s="9">
+        <v>162</v>
+      </c>
+      <c r="O18" s="9">
+        <v>5</v>
+      </c>
+      <c r="P18" s="8" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="13">
@@ -1351,19 +1483,33 @@
       <c r="F19" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="8"/>
+      <c r="G19" s="8" t="s">
+        <v>99</v>
+      </c>
       <c r="H19" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I19" s="14">
         <v>0</v>
       </c>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
+      <c r="J19" s="9">
+        <v>0</v>
+      </c>
+      <c r="K19" s="9">
+        <v>0</v>
+      </c>
+      <c r="L19" s="9">
+        <v>0</v>
+      </c>
+      <c r="M19" s="9">
+        <v>0</v>
+      </c>
+      <c r="N19" s="9">
+        <v>0</v>
+      </c>
+      <c r="O19" s="9">
+        <v>0</v>
+      </c>
       <c r="P19" s="8"/>
     </row>
     <row r="20" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1382,20 +1528,36 @@
       <c r="F20" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="G20" s="8"/>
+      <c r="G20" s="8" t="s">
+        <v>90</v>
+      </c>
       <c r="H20" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I20" s="14">
         <v>0</v>
       </c>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="8"/>
+      <c r="J20" s="9">
+        <v>135</v>
+      </c>
+      <c r="K20" s="9">
+        <v>5.73</v>
+      </c>
+      <c r="L20" s="9">
+        <v>14.13</v>
+      </c>
+      <c r="M20" s="9">
+        <v>145</v>
+      </c>
+      <c r="N20" s="9">
+        <v>162</v>
+      </c>
+      <c r="O20" s="9">
+        <v>5</v>
+      </c>
+      <c r="P20" s="8" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="21" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="5">
@@ -1413,20 +1575,36 @@
       <c r="F21" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="8"/>
+      <c r="G21" s="8" t="s">
+        <v>87</v>
+      </c>
       <c r="H21" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I21" s="6">
         <v>65</v>
       </c>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="8"/>
+      <c r="J21" s="9">
+        <v>65</v>
+      </c>
+      <c r="K21" s="9">
+        <v>4.5</v>
+      </c>
+      <c r="L21" s="9">
+        <v>11.52</v>
+      </c>
+      <c r="M21" s="9">
+        <v>156</v>
+      </c>
+      <c r="N21" s="9">
+        <v>169</v>
+      </c>
+      <c r="O21" s="9">
+        <v>5</v>
+      </c>
+      <c r="P21" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="22" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10">
@@ -2749,11 +2927,11 @@
       </c>
       <c r="D7" s="17">
         <f>SUMIFS(Log!$J$6:$J$61,Log!$D$6:$D$61,B7)</f>
-        <v>0</v>
+        <v>242</v>
       </c>
       <c r="E7" s="17">
         <f>SUMIFS(Log!$K$6:$K$61,Log!$D$6:$D$61,B7)</f>
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="F7" s="17" t="str">
         <f>IFERROR(AVERAGEIFS(Log!$O$6:$O$61,Log!$D$6:$D$61,B7,Log!$H$6:$H$61,"Done"),"")</f>
@@ -2770,11 +2948,11 @@
       </c>
       <c r="D8" s="17">
         <f>SUMIFS(Log!$J$6:$J$61,Log!$D$6:$D$61,B8)</f>
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E8" s="17">
         <f>SUMIFS(Log!$K$6:$K$61,Log!$D$6:$D$61,B8)</f>
-        <v>0</v>
+        <v>10.23</v>
       </c>
       <c r="F8" s="17" t="str">
         <f>IFERROR(AVERAGEIFS(Log!$O$6:$O$61,Log!$D$6:$D$61,B8,Log!$H$6:$H$61,"Done"),"")</f>
@@ -2896,11 +3074,11 @@
       </c>
       <c r="D14" s="19">
         <f>SUM(D6:D13)</f>
-        <v>380</v>
+        <v>822</v>
       </c>
       <c r="E14" s="19">
         <f>SUM(E6:E13)</f>
-        <v>22.650000000000002</v>
+        <v>46.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Training log for 18AUG26
</commit_message>
<xml_diff>
--- a/Marathon_Training_Log.xlsx
+++ b/Marathon_Training_Log.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Coursework\24-Git_Projects\02-Marathon_Training_Personal\Marathon_Training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psaptarshi\Downloads\Marathon_Training-main\Marathon_Training-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2328B193-606B-4AD8-8991-A385DDED014A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7369C00D-C106-4562-A2D6-7856CF8ACAE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
     <sheet name="Weekly Summary" sheetId="2" r:id="rId2"/>
     <sheet name="Session Guide" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="115">
   <si>
     <t>Marathon Training Log — Pre-Super Base</t>
   </si>
@@ -382,6 +382,12 @@
   </si>
   <si>
     <t>20lb max weight training with focus on squats.</t>
+  </si>
+  <si>
+    <t>10 min warmup + 45 min class + 30 min class with last 10 min in cooldown</t>
+  </si>
+  <si>
+    <t>Very slow running. Did hit some hills so heart rate spiked during that time. But mostly the heart rate was below 148 bpm.</t>
   </si>
 </sst>
 </file>
@@ -817,28 +823,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:P61"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="43.140625" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" customWidth="1"/>
-    <col min="4" max="4" width="3.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="43.1796875" customWidth="1"/>
+    <col min="3" max="3" width="4.81640625" customWidth="1"/>
+    <col min="4" max="4" width="3.81640625" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
     <col min="6" max="6" width="111" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" customWidth="1"/>
-    <col min="8" max="8" width="7.7109375" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" customWidth="1"/>
-    <col min="13" max="13" width="7.5703125" customWidth="1"/>
+    <col min="7" max="7" width="71.54296875" customWidth="1"/>
+    <col min="8" max="8" width="7.7265625" customWidth="1"/>
+    <col min="12" max="12" width="9.54296875" customWidth="1"/>
+    <col min="13" max="13" width="7.54296875" customWidth="1"/>
     <col min="14" max="14" width="8" customWidth="1"/>
-    <col min="15" max="15" width="7.140625" customWidth="1"/>
-    <col min="16" max="16" width="73.5703125" customWidth="1"/>
+    <col min="15" max="15" width="7.1796875" customWidth="1"/>
+    <col min="16" max="16" width="73.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:16" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:16" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -846,7 +852,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
@@ -893,7 +899,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="5">
         <v>46230</v>
       </c>
@@ -940,7 +946,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" ht="93.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="10">
         <v>46231</v>
       </c>
@@ -987,7 +993,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="13">
         <v>46232</v>
       </c>
@@ -1034,7 +1040,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="5">
         <v>46233</v>
       </c>
@@ -1081,7 +1087,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="10">
         <v>46234</v>
       </c>
@@ -1128,7 +1134,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="10">
         <v>46235</v>
       </c>
@@ -1175,7 +1181,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="13">
         <v>46236</v>
       </c>
@@ -1222,7 +1228,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="13">
         <v>46237</v>
       </c>
@@ -1269,7 +1275,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="5">
         <v>46238</v>
       </c>
@@ -1316,7 +1322,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="10">
         <v>46239</v>
       </c>
@@ -1363,7 +1369,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="13">
         <v>46240</v>
       </c>
@@ -1408,7 +1414,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="5">
         <v>46241</v>
       </c>
@@ -1453,7 +1459,7 @@
       </c>
       <c r="P17" s="8"/>
     </row>
-    <row r="18" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="10">
         <v>46242</v>
       </c>
@@ -1500,7 +1506,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="13">
         <v>46243</v>
       </c>
@@ -1545,7 +1551,7 @@
       </c>
       <c r="P19" s="8"/>
     </row>
-    <row r="20" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="13">
         <v>46244</v>
       </c>
@@ -1592,7 +1598,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5">
         <v>46245</v>
       </c>
@@ -1639,7 +1645,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10">
         <v>46246</v>
       </c>
@@ -1686,7 +1692,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="13">
         <v>46247</v>
       </c>
@@ -1731,7 +1737,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="24" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="5">
         <v>46248</v>
       </c>
@@ -1776,7 +1782,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10">
         <v>46249</v>
       </c>
@@ -1823,7 +1829,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="13">
         <v>46250</v>
       </c>
@@ -1870,7 +1876,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="27" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="13">
         <v>46251</v>
       </c>
@@ -1917,7 +1923,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="5">
         <v>46252</v>
       </c>
@@ -1933,22 +1939,38 @@
       <c r="F28" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G28" s="8"/>
+      <c r="G28" s="8" t="s">
+        <v>113</v>
+      </c>
       <c r="H28" s="9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I28" s="6">
         <v>65</v>
       </c>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="8"/>
-    </row>
-    <row r="29" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J28" s="9">
+        <v>70</v>
+      </c>
+      <c r="K28" s="9">
+        <v>5</v>
+      </c>
+      <c r="L28" s="9">
+        <v>14.3</v>
+      </c>
+      <c r="M28" s="9">
+        <v>132</v>
+      </c>
+      <c r="N28" s="9">
+        <v>158</v>
+      </c>
+      <c r="O28" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="P28" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="10">
         <v>46253</v>
       </c>
@@ -1979,7 +2001,7 @@
       <c r="O29" s="9"/>
       <c r="P29" s="8"/>
     </row>
-    <row r="30" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13">
         <v>46254</v>
       </c>
@@ -2010,7 +2032,7 @@
       <c r="O30" s="9"/>
       <c r="P30" s="8"/>
     </row>
-    <row r="31" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="5">
         <v>46255</v>
       </c>
@@ -2041,7 +2063,7 @@
       <c r="O31" s="9"/>
       <c r="P31" s="8"/>
     </row>
-    <row r="32" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="10">
         <v>46256</v>
       </c>
@@ -2072,7 +2094,7 @@
       <c r="O32" s="9"/>
       <c r="P32" s="8"/>
     </row>
-    <row r="33" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="13">
         <v>46257</v>
       </c>
@@ -2103,7 +2125,7 @@
       <c r="O33" s="9"/>
       <c r="P33" s="8"/>
     </row>
-    <row r="34" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="13">
         <v>46258</v>
       </c>
@@ -2134,7 +2156,7 @@
       <c r="O34" s="9"/>
       <c r="P34" s="8"/>
     </row>
-    <row r="35" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="5">
         <v>46259</v>
       </c>
@@ -2165,7 +2187,7 @@
       <c r="O35" s="9"/>
       <c r="P35" s="8"/>
     </row>
-    <row r="36" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="10">
         <v>46260</v>
       </c>
@@ -2196,7 +2218,7 @@
       <c r="O36" s="9"/>
       <c r="P36" s="8"/>
     </row>
-    <row r="37" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="13">
         <v>46261</v>
       </c>
@@ -2227,7 +2249,7 @@
       <c r="O37" s="9"/>
       <c r="P37" s="8"/>
     </row>
-    <row r="38" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="5">
         <v>46262</v>
       </c>
@@ -2258,7 +2280,7 @@
       <c r="O38" s="9"/>
       <c r="P38" s="8"/>
     </row>
-    <row r="39" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="10">
         <v>46263</v>
       </c>
@@ -2289,7 +2311,7 @@
       <c r="O39" s="9"/>
       <c r="P39" s="8"/>
     </row>
-    <row r="40" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="13">
         <v>46264</v>
       </c>
@@ -2320,7 +2342,7 @@
       <c r="O40" s="9"/>
       <c r="P40" s="8"/>
     </row>
-    <row r="41" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="13">
         <v>46265</v>
       </c>
@@ -2351,7 +2373,7 @@
       <c r="O41" s="9"/>
       <c r="P41" s="8"/>
     </row>
-    <row r="42" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="5">
         <v>46266</v>
       </c>
@@ -2382,7 +2404,7 @@
       <c r="O42" s="9"/>
       <c r="P42" s="8"/>
     </row>
-    <row r="43" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="10">
         <v>46267</v>
       </c>
@@ -2413,7 +2435,7 @@
       <c r="O43" s="9"/>
       <c r="P43" s="8"/>
     </row>
-    <row r="44" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="13">
         <v>46268</v>
       </c>
@@ -2444,7 +2466,7 @@
       <c r="O44" s="9"/>
       <c r="P44" s="8"/>
     </row>
-    <row r="45" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="5">
         <v>46269</v>
       </c>
@@ -2475,7 +2497,7 @@
       <c r="O45" s="9"/>
       <c r="P45" s="8"/>
     </row>
-    <row r="46" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="10">
         <v>46270</v>
       </c>
@@ -2506,7 +2528,7 @@
       <c r="O46" s="9"/>
       <c r="P46" s="8"/>
     </row>
-    <row r="47" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="13">
         <v>46271</v>
       </c>
@@ -2537,7 +2559,7 @@
       <c r="O47" s="9"/>
       <c r="P47" s="8"/>
     </row>
-    <row r="48" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="13">
         <v>46272</v>
       </c>
@@ -2568,7 +2590,7 @@
       <c r="O48" s="9"/>
       <c r="P48" s="8"/>
     </row>
-    <row r="49" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="5">
         <v>46273</v>
       </c>
@@ -2599,7 +2621,7 @@
       <c r="O49" s="9"/>
       <c r="P49" s="8"/>
     </row>
-    <row r="50" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="10">
         <v>46274</v>
       </c>
@@ -2630,7 +2652,7 @@
       <c r="O50" s="9"/>
       <c r="P50" s="8"/>
     </row>
-    <row r="51" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="13">
         <v>46275</v>
       </c>
@@ -2661,7 +2683,7 @@
       <c r="O51" s="9"/>
       <c r="P51" s="8"/>
     </row>
-    <row r="52" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="5">
         <v>46276</v>
       </c>
@@ -2692,7 +2714,7 @@
       <c r="O52" s="9"/>
       <c r="P52" s="8"/>
     </row>
-    <row r="53" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="10">
         <v>46277</v>
       </c>
@@ -2723,7 +2745,7 @@
       <c r="O53" s="9"/>
       <c r="P53" s="8"/>
     </row>
-    <row r="54" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="13">
         <v>46278</v>
       </c>
@@ -2754,7 +2776,7 @@
       <c r="O54" s="9"/>
       <c r="P54" s="8"/>
     </row>
-    <row r="55" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="13">
         <v>46279</v>
       </c>
@@ -2785,7 +2807,7 @@
       <c r="O55" s="9"/>
       <c r="P55" s="8"/>
     </row>
-    <row r="56" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="5">
         <v>46280</v>
       </c>
@@ -2816,7 +2838,7 @@
       <c r="O56" s="9"/>
       <c r="P56" s="8"/>
     </row>
-    <row r="57" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="10">
         <v>46281</v>
       </c>
@@ -2847,7 +2869,7 @@
       <c r="O57" s="9"/>
       <c r="P57" s="8"/>
     </row>
-    <row r="58" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="13">
         <v>46282</v>
       </c>
@@ -2878,7 +2900,7 @@
       <c r="O58" s="9"/>
       <c r="P58" s="8"/>
     </row>
-    <row r="59" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="5">
         <v>46283</v>
       </c>
@@ -2909,7 +2931,7 @@
       <c r="O59" s="9"/>
       <c r="P59" s="8"/>
     </row>
-    <row r="60" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="10">
         <v>46284</v>
       </c>
@@ -2940,7 +2962,7 @@
       <c r="O60" s="9"/>
       <c r="P60" s="8"/>
     </row>
-    <row r="61" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B61" s="13">
         <v>46285</v>
       </c>
@@ -2986,7 +3008,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:F14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -2994,17 +3016,17 @@
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="16" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
@@ -3021,7 +3043,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="17">
         <v>1</v>
       </c>
@@ -3042,7 +3064,7 @@
         <v>4.833333333333333</v>
       </c>
     </row>
-    <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="17">
         <v>2</v>
       </c>
@@ -3063,7 +3085,7 @@
         <v>3.75</v>
       </c>
     </row>
-    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="17">
         <v>3</v>
       </c>
@@ -3084,28 +3106,28 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="17">
         <v>4</v>
       </c>
       <c r="C9" s="17">
         <f>COUNTIFS(Log!$D$6:$D$61,B9,Log!$H$6:$H$61,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="17">
         <f>SUMIFS(Log!$J$6:$J$61,Log!$D$6:$D$61,B9)</f>
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="E9" s="17">
         <f>SUMIFS(Log!$K$6:$K$61,Log!$D$6:$D$61,B9)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F9" s="17">
         <f>IFERROR(AVERAGEIFS(Log!$O$6:$O$61,Log!$D$6:$D$61,B9,Log!$H$6:$H$61,"Done"),"")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="17">
         <v>5</v>
       </c>
@@ -3126,7 +3148,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="17">
         <v>6</v>
       </c>
@@ -3147,7 +3169,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="17">
         <v>7</v>
       </c>
@@ -3168,7 +3190,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="17">
         <v>8</v>
       </c>
@@ -3189,21 +3211,21 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>58</v>
       </c>
       <c r="C14" s="19">
         <f>SUM(C6:C13)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D14" s="19">
         <f>SUM(D6:D13)</f>
-        <v>1085</v>
+        <v>1155</v>
       </c>
       <c r="E14" s="19">
         <f>SUM(E6:E13)</f>
-        <v>59.17</v>
+        <v>64.17</v>
       </c>
     </row>
   </sheetData>
@@ -3215,23 +3237,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="16" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="20" t="s">
         <v>61</v>
       </c>
@@ -3239,7 +3261,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="20" t="s">
         <v>63</v>
       </c>
@@ -3247,7 +3269,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="20" t="s">
         <v>65</v>
       </c>
@@ -3255,7 +3277,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:3" ht="70.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>67</v>
       </c>
@@ -3263,7 +3285,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:3" ht="77.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="20" t="s">
         <v>69</v>
       </c>
@@ -3271,7 +3293,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="20" t="s">
         <v>71</v>
       </c>
@@ -3279,7 +3301,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="20" t="s">
         <v>73</v>
       </c>

</xml_diff>

<commit_message>
Added log for 19AUG26
</commit_message>
<xml_diff>
--- a/Marathon_Training_Log.xlsx
+++ b/Marathon_Training_Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psaptarshi\Downloads\Marathon_Training-main\Marathon_Training-main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Coursework\24-Git_Projects\02-Marathon_Training_Personal\Marathon_Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7369C00D-C106-4562-A2D6-7856CF8ACAE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4306A78F-BF6D-494A-8191-D778F9250375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="117">
   <si>
     <t>Marathon Training Log — Pre-Super Base</t>
   </si>
@@ -388,6 +388,18 @@
   </si>
   <si>
     <t>Very slow running. Did hit some hills so heart rate spiked during that time. But mostly the heart rate was below 148 bpm.</t>
+  </si>
+  <si>
+    <t>15 min warmup + 45 min Tempo Run with Becs Gentry + 10 min coolodown</t>
+  </si>
+  <si>
+    <t>15 min very slow run at 3 miles/hr
+Followed by the set.
+1st set: Ran at 6 miles/hr with 0.5% incline. Not terrible, but found needing more and more time to recover heartrate back to around 130s. So dropped. RPE 6.5
+2nd set: Ran at 5.8 miles/hr with 0.5% incline. Felt better. RPE 6.5
+3rd set: Ran at 5.8 miles/hr with 0% incline. Stress felt similar to RPE 6.5
+After each run, jogged at 3 miles/hr for 2min 20 sec.
+Between each set jogged at 3 miles/hr for almost 4 min.</t>
   </si>
 </sst>
 </file>
@@ -823,28 +835,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:P61"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="43.1796875" customWidth="1"/>
-    <col min="3" max="3" width="4.81640625" customWidth="1"/>
-    <col min="4" max="4" width="3.81640625" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="2" max="2" width="43.140625" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" customWidth="1"/>
+    <col min="4" max="4" width="3.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
     <col min="6" max="6" width="111" customWidth="1"/>
-    <col min="7" max="7" width="71.54296875" customWidth="1"/>
-    <col min="8" max="8" width="7.7265625" customWidth="1"/>
-    <col min="12" max="12" width="9.54296875" customWidth="1"/>
-    <col min="13" max="13" width="7.54296875" customWidth="1"/>
+    <col min="7" max="7" width="71.5703125" customWidth="1"/>
+    <col min="8" max="8" width="7.7109375" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" customWidth="1"/>
+    <col min="13" max="13" width="7.5703125" customWidth="1"/>
     <col min="14" max="14" width="8" customWidth="1"/>
-    <col min="15" max="15" width="7.1796875" customWidth="1"/>
-    <col min="16" max="16" width="73.54296875" customWidth="1"/>
+    <col min="15" max="15" width="7.140625" customWidth="1"/>
+    <col min="16" max="16" width="73.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:16" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:16" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -852,7 +864,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
@@ -899,7 +911,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5">
         <v>46230</v>
       </c>
@@ -946,7 +958,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="93.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:16" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="10">
         <v>46231</v>
       </c>
@@ -993,7 +1005,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="13">
         <v>46232</v>
       </c>
@@ -1040,7 +1052,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
         <v>46233</v>
       </c>
@@ -1087,7 +1099,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10">
         <v>46234</v>
       </c>
@@ -1134,7 +1146,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="10">
         <v>46235</v>
       </c>
@@ -1181,7 +1193,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="13">
         <v>46236</v>
       </c>
@@ -1228,7 +1240,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="13">
         <v>46237</v>
       </c>
@@ -1275,7 +1287,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5">
         <v>46238</v>
       </c>
@@ -1322,7 +1334,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="10">
         <v>46239</v>
       </c>
@@ -1369,7 +1381,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="13">
         <v>46240</v>
       </c>
@@ -1414,7 +1426,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="5">
         <v>46241</v>
       </c>
@@ -1459,7 +1471,7 @@
       </c>
       <c r="P17" s="8"/>
     </row>
-    <row r="18" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="10">
         <v>46242</v>
       </c>
@@ -1506,7 +1518,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="13">
         <v>46243</v>
       </c>
@@ -1551,7 +1563,7 @@
       </c>
       <c r="P19" s="8"/>
     </row>
-    <row r="20" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="13">
         <v>46244</v>
       </c>
@@ -1598,7 +1610,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="5">
         <v>46245</v>
       </c>
@@ -1645,7 +1657,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10">
         <v>46246</v>
       </c>
@@ -1692,7 +1704,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="13">
         <v>46247</v>
       </c>
@@ -1737,7 +1749,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="24" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="5">
         <v>46248</v>
       </c>
@@ -1782,7 +1794,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10">
         <v>46249</v>
       </c>
@@ -1829,7 +1841,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="13">
         <v>46250</v>
       </c>
@@ -1876,7 +1888,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="27" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="13">
         <v>46251</v>
       </c>
@@ -1923,7 +1935,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="5">
         <v>46252</v>
       </c>
@@ -1970,7 +1982,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="29" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:16" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="10">
         <v>46253</v>
       </c>
@@ -1986,22 +1998,38 @@
       <c r="F29" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G29" s="8"/>
+      <c r="G29" s="8" t="s">
+        <v>115</v>
+      </c>
       <c r="H29" s="9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I29" s="11">
         <v>57</v>
       </c>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
-      <c r="L29" s="9"/>
-      <c r="M29" s="9"/>
-      <c r="N29" s="9"/>
-      <c r="O29" s="9"/>
-      <c r="P29" s="8"/>
-    </row>
-    <row r="30" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J29" s="9">
+        <v>70</v>
+      </c>
+      <c r="K29" s="9">
+        <v>4</v>
+      </c>
+      <c r="L29" s="9">
+        <v>18.29</v>
+      </c>
+      <c r="M29" s="9">
+        <v>144</v>
+      </c>
+      <c r="N29" s="9">
+        <v>172</v>
+      </c>
+      <c r="O29" s="9">
+        <v>6.5</v>
+      </c>
+      <c r="P29" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13">
         <v>46254</v>
       </c>
@@ -2032,7 +2060,7 @@
       <c r="O30" s="9"/>
       <c r="P30" s="8"/>
     </row>
-    <row r="31" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="5">
         <v>46255</v>
       </c>
@@ -2063,7 +2091,7 @@
       <c r="O31" s="9"/>
       <c r="P31" s="8"/>
     </row>
-    <row r="32" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="10">
         <v>46256</v>
       </c>
@@ -2094,7 +2122,7 @@
       <c r="O32" s="9"/>
       <c r="P32" s="8"/>
     </row>
-    <row r="33" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="13">
         <v>46257</v>
       </c>
@@ -2125,7 +2153,7 @@
       <c r="O33" s="9"/>
       <c r="P33" s="8"/>
     </row>
-    <row r="34" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="13">
         <v>46258</v>
       </c>
@@ -2156,7 +2184,7 @@
       <c r="O34" s="9"/>
       <c r="P34" s="8"/>
     </row>
-    <row r="35" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="5">
         <v>46259</v>
       </c>
@@ -2187,7 +2215,7 @@
       <c r="O35" s="9"/>
       <c r="P35" s="8"/>
     </row>
-    <row r="36" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="10">
         <v>46260</v>
       </c>
@@ -2218,7 +2246,7 @@
       <c r="O36" s="9"/>
       <c r="P36" s="8"/>
     </row>
-    <row r="37" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="13">
         <v>46261</v>
       </c>
@@ -2249,7 +2277,7 @@
       <c r="O37" s="9"/>
       <c r="P37" s="8"/>
     </row>
-    <row r="38" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="5">
         <v>46262</v>
       </c>
@@ -2280,7 +2308,7 @@
       <c r="O38" s="9"/>
       <c r="P38" s="8"/>
     </row>
-    <row r="39" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="10">
         <v>46263</v>
       </c>
@@ -2311,7 +2339,7 @@
       <c r="O39" s="9"/>
       <c r="P39" s="8"/>
     </row>
-    <row r="40" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="13">
         <v>46264</v>
       </c>
@@ -2342,7 +2370,7 @@
       <c r="O40" s="9"/>
       <c r="P40" s="8"/>
     </row>
-    <row r="41" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="13">
         <v>46265</v>
       </c>
@@ -2373,7 +2401,7 @@
       <c r="O41" s="9"/>
       <c r="P41" s="8"/>
     </row>
-    <row r="42" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="5">
         <v>46266</v>
       </c>
@@ -2404,7 +2432,7 @@
       <c r="O42" s="9"/>
       <c r="P42" s="8"/>
     </row>
-    <row r="43" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="10">
         <v>46267</v>
       </c>
@@ -2435,7 +2463,7 @@
       <c r="O43" s="9"/>
       <c r="P43" s="8"/>
     </row>
-    <row r="44" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="13">
         <v>46268</v>
       </c>
@@ -2466,7 +2494,7 @@
       <c r="O44" s="9"/>
       <c r="P44" s="8"/>
     </row>
-    <row r="45" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="5">
         <v>46269</v>
       </c>
@@ -2497,7 +2525,7 @@
       <c r="O45" s="9"/>
       <c r="P45" s="8"/>
     </row>
-    <row r="46" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="10">
         <v>46270</v>
       </c>
@@ -2528,7 +2556,7 @@
       <c r="O46" s="9"/>
       <c r="P46" s="8"/>
     </row>
-    <row r="47" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="13">
         <v>46271</v>
       </c>
@@ -2559,7 +2587,7 @@
       <c r="O47" s="9"/>
       <c r="P47" s="8"/>
     </row>
-    <row r="48" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="13">
         <v>46272</v>
       </c>
@@ -2590,7 +2618,7 @@
       <c r="O48" s="9"/>
       <c r="P48" s="8"/>
     </row>
-    <row r="49" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="5">
         <v>46273</v>
       </c>
@@ -2621,7 +2649,7 @@
       <c r="O49" s="9"/>
       <c r="P49" s="8"/>
     </row>
-    <row r="50" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="10">
         <v>46274</v>
       </c>
@@ -2652,7 +2680,7 @@
       <c r="O50" s="9"/>
       <c r="P50" s="8"/>
     </row>
-    <row r="51" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="13">
         <v>46275</v>
       </c>
@@ -2683,7 +2711,7 @@
       <c r="O51" s="9"/>
       <c r="P51" s="8"/>
     </row>
-    <row r="52" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="5">
         <v>46276</v>
       </c>
@@ -2714,7 +2742,7 @@
       <c r="O52" s="9"/>
       <c r="P52" s="8"/>
     </row>
-    <row r="53" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="10">
         <v>46277</v>
       </c>
@@ -2745,7 +2773,7 @@
       <c r="O53" s="9"/>
       <c r="P53" s="8"/>
     </row>
-    <row r="54" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="13">
         <v>46278</v>
       </c>
@@ -2776,7 +2804,7 @@
       <c r="O54" s="9"/>
       <c r="P54" s="8"/>
     </row>
-    <row r="55" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="13">
         <v>46279</v>
       </c>
@@ -2807,7 +2835,7 @@
       <c r="O55" s="9"/>
       <c r="P55" s="8"/>
     </row>
-    <row r="56" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="5">
         <v>46280</v>
       </c>
@@ -2838,7 +2866,7 @@
       <c r="O56" s="9"/>
       <c r="P56" s="8"/>
     </row>
-    <row r="57" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="10">
         <v>46281</v>
       </c>
@@ -2869,7 +2897,7 @@
       <c r="O57" s="9"/>
       <c r="P57" s="8"/>
     </row>
-    <row r="58" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="13">
         <v>46282</v>
       </c>
@@ -2900,7 +2928,7 @@
       <c r="O58" s="9"/>
       <c r="P58" s="8"/>
     </row>
-    <row r="59" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="5">
         <v>46283</v>
       </c>
@@ -2931,7 +2959,7 @@
       <c r="O59" s="9"/>
       <c r="P59" s="8"/>
     </row>
-    <row r="60" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="10">
         <v>46284</v>
       </c>
@@ -2962,7 +2990,7 @@
       <c r="O60" s="9"/>
       <c r="P60" s="8"/>
     </row>
-    <row r="61" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="13">
         <v>46285</v>
       </c>
@@ -3008,7 +3036,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:F14"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -3016,17 +3044,17 @@
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="16" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
@@ -3043,7 +3071,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="17">
         <v>1</v>
       </c>
@@ -3064,7 +3092,7 @@
         <v>4.833333333333333</v>
       </c>
     </row>
-    <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="17">
         <v>2</v>
       </c>
@@ -3085,7 +3113,7 @@
         <v>3.75</v>
       </c>
     </row>
-    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="17">
         <v>3</v>
       </c>
@@ -3106,28 +3134,28 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="17">
         <v>4</v>
       </c>
       <c r="C9" s="17">
         <f>COUNTIFS(Log!$D$6:$D$61,B9,Log!$H$6:$H$61,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="17">
         <f>SUMIFS(Log!$J$6:$J$61,Log!$D$6:$D$61,B9)</f>
-        <v>102</v>
+        <v>172</v>
       </c>
       <c r="E9" s="17">
         <f>SUMIFS(Log!$K$6:$K$61,Log!$D$6:$D$61,B9)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F9" s="17">
         <f>IFERROR(AVERAGEIFS(Log!$O$6:$O$61,Log!$D$6:$D$61,B9,Log!$H$6:$H$61,"Done"),"")</f>
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>4.333333333333333</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="17">
         <v>5</v>
       </c>
@@ -3148,7 +3176,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="17">
         <v>6</v>
       </c>
@@ -3169,7 +3197,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="17">
         <v>7</v>
       </c>
@@ -3190,7 +3218,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="17">
         <v>8</v>
       </c>
@@ -3211,21 +3239,21 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
         <v>58</v>
       </c>
       <c r="C14" s="19">
         <f>SUM(C6:C13)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D14" s="19">
         <f>SUM(D6:D13)</f>
-        <v>1155</v>
+        <v>1225</v>
       </c>
       <c r="E14" s="19">
         <f>SUM(E6:E13)</f>
-        <v>64.17</v>
+        <v>68.17</v>
       </c>
     </row>
   </sheetData>
@@ -3237,23 +3265,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="16" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="20" t="s">
         <v>61</v>
       </c>
@@ -3261,7 +3289,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
         <v>63</v>
       </c>
@@ -3269,7 +3297,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="20" t="s">
         <v>65</v>
       </c>
@@ -3277,7 +3305,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="70.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>67</v>
       </c>
@@ -3285,7 +3313,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="77.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="20" t="s">
         <v>69</v>
       </c>
@@ -3293,7 +3321,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="20" t="s">
         <v>71</v>
       </c>
@@ -3301,7 +3329,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="20" t="s">
         <v>73</v>
       </c>

</xml_diff>